<commit_message>
Minor changes in auth
>Colocar o back na página de reset
>Ainda há erros no NgModule de LoginPage
>Testar domínio de email
>Correção do placeholder de reset de senha e no botão
>Reset de senha com sucesso
</commit_message>
<xml_diff>
--- a/PENDÊNCIAS APP.xlsx
+++ b/PENDÊNCIAS APP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="19330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iago Rodriguez\Documents\GitHub\ProjetoDCE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C444023-E516-4CDE-AAEE-3529CF335C1F}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10C54DBF-18EE-49F0-B671-8087CB75EC34}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9075" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tarefas" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="73">
   <si>
     <t xml:space="preserve">
  Pendências</t>
@@ -201,6 +201,48 @@
   </si>
   <si>
     <t>https://firebase.google.com/products/cloud-messaging/?authuser=0</t>
+  </si>
+  <si>
+    <t>Para verificar seu domínio, adicione os registros DNS a seguir a seu registro de domínio.</t>
+  </si>
+  <si>
+    <t>Host</t>
+  </si>
+  <si>
+    <t>Tipo</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>dcefacamp.com</t>
+  </si>
+  <si>
+    <t>TXT</t>
+  </si>
+  <si>
+    <t>v=spf1 include:_spf.firebasemail.com ~all</t>
+  </si>
+  <si>
+    <t>firebase=dcechecker</t>
+  </si>
+  <si>
+    <t>firebase1._domainkey.dcefacamp.com</t>
+  </si>
+  <si>
+    <t>CNAME</t>
+  </si>
+  <si>
+    <t>mail-dcefacamp-com.dkim1._domainkey.firebasemail.com.</t>
+  </si>
+  <si>
+    <t>firebase2._domainkey.dcefacamp.com</t>
+  </si>
+  <si>
+    <t>mail-dcefacamp-com.dkim2._domainkey.firebasemail.com.</t>
+  </si>
+  <si>
+    <t>Verificar domínio</t>
   </si>
 </sst>
 </file>
@@ -211,7 +253,7 @@
     <numFmt numFmtId="164" formatCode="d&quot;/&quot;m"/>
     <numFmt numFmtId="165" formatCode="dd&quot;/&quot;mm"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -279,8 +321,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -297,6 +351,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF0D904F"/>
         <bgColor rgb="FF0D904F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -355,7 +421,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -423,10 +489,32 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -782,22 +870,22 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:E48"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" customWidth="1"/>
     <col min="3" max="3" width="140" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="52.5" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
+      <c r="B1" s="29"/>
       <c r="C1" s="1" t="str">
         <f>CONCATENATE(COUNTA($A$4:$A$34), "/", COUNTA($C$4:$C$34), " concluído  ")</f>
-        <v xml:space="preserve">5/31 concluído  </v>
+        <v xml:space="preserve">6/31 concluído  </v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="6" customHeight="1">
@@ -888,7 +976,9 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="26.25" customHeight="1">
-      <c r="A10" s="10"/>
+      <c r="A10" s="10" t="s">
+        <v>37</v>
+      </c>
       <c r="B10" s="11"/>
       <c r="C10" s="20" t="s">
         <v>11</v>
@@ -1109,19 +1199,89 @@
         <v>45</v>
       </c>
     </row>
-    <row r="36" spans="1:5" s="25" customFormat="1" ht="22.5" customHeight="1">
+    <row r="36" spans="1:5" s="27" customFormat="1" ht="22.5" customHeight="1">
       <c r="A36" s="16"/>
       <c r="B36" s="17"/>
       <c r="C36" s="15" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" s="25" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A37" s="16"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="E36" s="24" t="s">
+      <c r="E37" s="24" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="15.75" customHeight="1">
-      <c r="C39" s="24" t="s">
+    <row r="40" spans="1:5" ht="15.75" customHeight="1">
+      <c r="C40" s="24" t="s">
         <v>57</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="15.75" customHeight="1">
+      <c r="C41" s="30"/>
+    </row>
+    <row r="43" spans="1:5" ht="15.75" customHeight="1">
+      <c r="C43" s="31" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="15.75" customHeight="1">
+      <c r="C44" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="D44" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="E44" s="32" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="15.75" customHeight="1">
+      <c r="C45" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="D45" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="E45" s="33" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="15.75" customHeight="1">
+      <c r="C46" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="D46" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="E46" s="33" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="15.75" customHeight="1">
+      <c r="C47" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="D47" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="E47" s="33" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="15.75" customHeight="1">
+      <c r="C48" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D48" s="36" t="s">
+        <v>68</v>
+      </c>
+      <c r="E48" s="35" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1129,7 +1289,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A4:XFD14 A15:B16 D15:XFD16 C15 A17:XFD35">
+  <conditionalFormatting sqref="A4:XFD14 A15:B16 D15:XFD16 C15 A17:XFD36">
     <cfRule type="expression" dxfId="2" priority="2">
       <formula>NOT(ISBLANK($A4))</formula>
     </cfRule>
@@ -1139,9 +1299,9 @@
       <formula>NOT(ISBLANK($A15))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A36:XFD36">
+  <conditionalFormatting sqref="A37:XFD37">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>NOT(ISBLANK($A36))</formula>
+      <formula>NOT(ISBLANK($A37))</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>

</xml_diff>